<commit_message>
Cotacoes CEAGESP - coleta de 04/08/2026 23:11
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historico" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Historico" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$36</definedName>
@@ -539,7 +539,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:34</t>
+          <t>04/08/2026 23:11:23</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:34</t>
+          <t>04/08/2026 23:11:23</t>
         </is>
       </c>
     </row>
@@ -627,7 +627,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:34</t>
+          <t>04/08/2026 23:11:23</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:34</t>
+          <t>04/08/2026 23:11:23</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:34</t>
+          <t>04/08/2026 23:11:23</t>
         </is>
       </c>
     </row>
@@ -759,7 +759,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:34</t>
+          <t>04/08/2026 23:11:23</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:37</t>
+          <t>04/08/2026 23:11:26</t>
         </is>
       </c>
     </row>
@@ -847,7 +847,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:37</t>
+          <t>04/08/2026 23:11:26</t>
         </is>
       </c>
     </row>
@@ -891,7 +891,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:40</t>
+          <t>04/08/2026 23:11:29</t>
         </is>
       </c>
     </row>
@@ -935,7 +935,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:40</t>
+          <t>04/08/2026 23:11:29</t>
         </is>
       </c>
     </row>
@@ -979,7 +979,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:40</t>
+          <t>04/08/2026 23:11:29</t>
         </is>
       </c>
     </row>
@@ -1023,7 +1023,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:40</t>
+          <t>04/08/2026 23:11:29</t>
         </is>
       </c>
     </row>
@@ -1067,7 +1067,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:40</t>
+          <t>04/08/2026 23:11:29</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:40</t>
+          <t>04/08/2026 23:11:29</t>
         </is>
       </c>
     </row>
@@ -1155,7 +1155,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:43</t>
+          <t>04/08/2026 23:11:32</t>
         </is>
       </c>
     </row>
@@ -1199,7 +1199,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:43</t>
+          <t>04/08/2026 23:11:32</t>
         </is>
       </c>
     </row>
@@ -1243,7 +1243,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:43</t>
+          <t>04/08/2026 23:11:32</t>
         </is>
       </c>
     </row>
@@ -1287,7 +1287,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:43</t>
+          <t>04/08/2026 23:11:32</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1331,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:43</t>
+          <t>04/08/2026 23:11:32</t>
         </is>
       </c>
     </row>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:43</t>
+          <t>04/08/2026 23:11:32</t>
         </is>
       </c>
     </row>
@@ -1419,7 +1419,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:45</t>
+          <t>04/08/2026 23:11:35</t>
         </is>
       </c>
     </row>
@@ -1463,7 +1463,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:45</t>
+          <t>04/08/2026 23:11:35</t>
         </is>
       </c>
     </row>
@@ -1507,7 +1507,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:45</t>
+          <t>04/08/2026 23:11:35</t>
         </is>
       </c>
     </row>
@@ -1551,7 +1551,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:48</t>
+          <t>04/08/2026 23:11:38</t>
         </is>
       </c>
     </row>
@@ -1595,7 +1595,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:48</t>
+          <t>04/08/2026 23:11:38</t>
         </is>
       </c>
     </row>
@@ -1639,7 +1639,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:48</t>
+          <t>04/08/2026 23:11:38</t>
         </is>
       </c>
     </row>
@@ -1683,7 +1683,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:48</t>
+          <t>04/08/2026 23:11:38</t>
         </is>
       </c>
     </row>
@@ -1727,7 +1727,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:48</t>
+          <t>04/08/2026 23:11:38</t>
         </is>
       </c>
     </row>
@@ -1771,7 +1771,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:48</t>
+          <t>04/08/2026 23:11:38</t>
         </is>
       </c>
     </row>
@@ -1815,7 +1815,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:51</t>
+          <t>04/08/2026 23:11:41</t>
         </is>
       </c>
     </row>
@@ -1859,7 +1859,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:51</t>
+          <t>04/08/2026 23:11:41</t>
         </is>
       </c>
     </row>
@@ -1903,7 +1903,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:51</t>
+          <t>04/08/2026 23:11:41</t>
         </is>
       </c>
     </row>
@@ -1947,7 +1947,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:51</t>
+          <t>04/08/2026 23:11:41</t>
         </is>
       </c>
     </row>
@@ -1991,7 +1991,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:51</t>
+          <t>04/08/2026 23:11:41</t>
         </is>
       </c>
     </row>
@@ -2035,7 +2035,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:51</t>
+          <t>04/08/2026 23:11:41</t>
         </is>
       </c>
     </row>
@@ -2158,7 +2158,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:51</t>
+          <t>04/08/2026 23:11:41</t>
         </is>
       </c>
     </row>
@@ -2202,7 +2202,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:51</t>
+          <t>04/08/2026 23:11:41</t>
         </is>
       </c>
     </row>
@@ -2246,7 +2246,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:51</t>
+          <t>04/08/2026 23:11:41</t>
         </is>
       </c>
     </row>
@@ -2290,7 +2290,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:51</t>
+          <t>04/08/2026 23:11:41</t>
         </is>
       </c>
     </row>
@@ -2334,7 +2334,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:51</t>
+          <t>04/08/2026 23:11:41</t>
         </is>
       </c>
     </row>
@@ -2378,7 +2378,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>04/08/2026 16:15:51</t>
+          <t>04/08/2026 23:11:41</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cotacoes CEAGESP - coleta de 04/08/2026 23:40
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -1815,7 +1815,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>04/08/2026 23:11:41</t>
+          <t>04/08/2026 23:40:10</t>
         </is>
       </c>
     </row>
@@ -1859,7 +1859,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>04/08/2026 23:11:41</t>
+          <t>04/08/2026 23:40:10</t>
         </is>
       </c>
     </row>
@@ -1903,7 +1903,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>04/08/2026 23:11:41</t>
+          <t>04/08/2026 23:40:10</t>
         </is>
       </c>
     </row>
@@ -1947,7 +1947,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>04/08/2026 23:11:41</t>
+          <t>04/08/2026 23:40:10</t>
         </is>
       </c>
     </row>
@@ -1991,7 +1991,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>04/08/2026 23:11:41</t>
+          <t>04/08/2026 23:40:10</t>
         </is>
       </c>
     </row>
@@ -2035,7 +2035,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>04/08/2026 23:11:41</t>
+          <t>04/08/2026 23:40:10</t>
         </is>
       </c>
     </row>
@@ -2158,7 +2158,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>04/08/2026 23:11:41</t>
+          <t>04/08/2026 23:40:10</t>
         </is>
       </c>
     </row>
@@ -2202,7 +2202,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>04/08/2026 23:11:41</t>
+          <t>04/08/2026 23:40:10</t>
         </is>
       </c>
     </row>
@@ -2246,7 +2246,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>04/08/2026 23:11:41</t>
+          <t>04/08/2026 23:40:10</t>
         </is>
       </c>
     </row>
@@ -2290,7 +2290,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>04/08/2026 23:11:41</t>
+          <t>04/08/2026 23:40:10</t>
         </is>
       </c>
     </row>
@@ -2334,7 +2334,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>04/08/2026 23:11:41</t>
+          <t>04/08/2026 23:40:10</t>
         </is>
       </c>
     </row>
@@ -2378,7 +2378,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>04/08/2026 23:11:41</t>
+          <t>04/08/2026 23:40:10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Regera planilha e pagina apos o rebase
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -14927,7 +14927,7 @@
       </c>
       <c r="J329" t="inlineStr">
         <is>
-          <t>04/08/2026 23:11:41</t>
+          <t>04/08/2026 23:40:10</t>
         </is>
       </c>
     </row>
@@ -14971,7 +14971,7 @@
       </c>
       <c r="J330" t="inlineStr">
         <is>
-          <t>04/08/2026 23:11:41</t>
+          <t>04/08/2026 23:40:10</t>
         </is>
       </c>
     </row>
@@ -15015,7 +15015,7 @@
       </c>
       <c r="J331" t="inlineStr">
         <is>
-          <t>04/08/2026 23:11:41</t>
+          <t>04/08/2026 23:40:10</t>
         </is>
       </c>
     </row>
@@ -15059,7 +15059,7 @@
       </c>
       <c r="J332" t="inlineStr">
         <is>
-          <t>04/08/2026 23:11:41</t>
+          <t>04/08/2026 23:40:10</t>
         </is>
       </c>
     </row>
@@ -15103,7 +15103,7 @@
       </c>
       <c r="J333" t="inlineStr">
         <is>
-          <t>04/08/2026 23:11:41</t>
+          <t>04/08/2026 23:40:10</t>
         </is>
       </c>
     </row>
@@ -15147,7 +15147,7 @@
       </c>
       <c r="J334" t="inlineStr">
         <is>
-          <t>04/08/2026 23:11:41</t>
+          <t>04/08/2026 23:40:10</t>
         </is>
       </c>
     </row>
@@ -15270,7 +15270,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>04/08/2026 23:11:41</t>
+          <t>04/08/2026 23:40:10</t>
         </is>
       </c>
     </row>
@@ -15314,7 +15314,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>04/08/2026 23:11:41</t>
+          <t>04/08/2026 23:40:10</t>
         </is>
       </c>
     </row>
@@ -15358,7 +15358,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>04/08/2026 23:11:41</t>
+          <t>04/08/2026 23:40:10</t>
         </is>
       </c>
     </row>
@@ -15402,7 +15402,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>04/08/2026 23:11:41</t>
+          <t>04/08/2026 23:40:10</t>
         </is>
       </c>
     </row>
@@ -15446,7 +15446,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>04/08/2026 23:11:41</t>
+          <t>04/08/2026 23:40:10</t>
         </is>
       </c>
     </row>
@@ -15490,7 +15490,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>04/08/2026 23:11:41</t>
+          <t>04/08/2026 23:40:10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cotacoes CEAGESP - coleta de 06/08/2026 10:51
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historico" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Historico" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$334</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$339</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J334"/>
+  <dimension ref="A1:J339"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -15151,8 +15151,228 @@
         </is>
       </c>
     </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>05/08/2026</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>FILE DE TILAPIA</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F335" s="2" t="n">
+        <v>42.27</v>
+      </c>
+      <c r="G335" s="2" t="n">
+        <v>42.84</v>
+      </c>
+      <c r="H335" s="2" t="n">
+        <v>43.41</v>
+      </c>
+      <c r="I335" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J335" t="inlineStr">
+        <is>
+          <t>06/08/2026 10:51:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>05/08/2026</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>PINTADO</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F336" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G336" s="2" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="H336" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="I336" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J336" t="inlineStr">
+        <is>
+          <t>06/08/2026 10:51:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>05/08/2026</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>TAMBAQUI</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F337" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="G337" s="2" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="H337" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="I337" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J337" t="inlineStr">
+        <is>
+          <t>06/08/2026 10:51:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>05/08/2026</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F338" s="2" t="n">
+        <v>11.93</v>
+      </c>
+      <c r="G338" s="2" t="n">
+        <v>12.22</v>
+      </c>
+      <c r="H338" s="2" t="n">
+        <v>12.45</v>
+      </c>
+      <c r="I338" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J338" t="inlineStr">
+        <is>
+          <t>06/08/2026 10:51:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>05/08/2026</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>TRUTA</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F339" s="2" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="G339" s="2" t="n">
+        <v>38.25</v>
+      </c>
+      <c r="H339" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="I339" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J339" t="inlineStr">
+        <is>
+          <t>06/08/2026 10:51:43</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J334"/>
+  <autoFilter ref="A1:J339"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -15163,7 +15383,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -15233,7 +15453,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>03/08/2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -15257,27 +15477,27 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>42.52</v>
+        <v>42.27</v>
       </c>
       <c r="G2" s="2" t="n">
+        <v>42.84</v>
+      </c>
+      <c r="H2" s="2" t="n">
         <v>43.41</v>
       </c>
-      <c r="H2" s="2" t="n">
-        <v>44.34</v>
-      </c>
       <c r="I2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>04/08/2026 23:40:10</t>
+          <t>06/08/2026 10:51:43</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>03/08/2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -15287,7 +15507,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>PANGASIUS</t>
+          <t>PINTADO</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -15301,27 +15521,27 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>9.800000000000001</v>
+        <v>25</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>9.9</v>
+        <v>25.5</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>04/08/2026 23:40:10</t>
+          <t>06/08/2026 10:51:43</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>03/08/2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -15331,7 +15551,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>PINTADO</t>
+          <t>TAMBAQUI</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -15345,27 +15565,27 @@
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>25.5</v>
+        <v>12</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>26</v>
+        <v>12.5</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>26.5</v>
+        <v>13</v>
       </c>
       <c r="I4" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>04/08/2026 23:40:10</t>
+          <t>06/08/2026 10:51:43</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>03/08/2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -15375,7 +15595,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>TAMBAQUI</t>
+          <t>TILÁPIA</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -15389,27 +15609,27 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>13</v>
+        <v>11.93</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>13.3</v>
+        <v>12.22</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>13.5</v>
+        <v>12.45</v>
       </c>
       <c r="I5" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>04/08/2026 23:40:10</t>
+          <t>06/08/2026 10:51:43</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>03/08/2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -15419,7 +15639,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>TILÁPIA</t>
+          <t>TRUTA</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -15433,69 +15653,25 @@
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>11.83</v>
+        <v>37.5</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>12.11</v>
+        <v>38.25</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>12.34</v>
+        <v>39</v>
       </c>
       <c r="I6" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>04/08/2026 23:40:10</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>03/08/2026</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>PESCADOS</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>TRUTA</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="n">
-        <v>38</v>
-      </c>
-      <c r="G7" s="2" t="n">
-        <v>38.5</v>
-      </c>
-      <c r="H7" s="2" t="n">
-        <v>39</v>
-      </c>
-      <c r="I7" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>04/08/2026 23:40:10</t>
+          <t>06/08/2026 10:51:43</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J7"/>
+  <autoFilter ref="A1:J6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Cotacoes CEAGESP - coleta de 09/08/2026 19:36
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$339</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$344</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J339"/>
+  <dimension ref="A1:J344"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -15371,8 +15371,228 @@
         </is>
       </c>
     </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>07/08/2026</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>FILE DE TILAPIA</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F340" s="2" t="n">
+        <v>42.61</v>
+      </c>
+      <c r="G340" s="2" t="n">
+        <v>43.48</v>
+      </c>
+      <c r="H340" s="2" t="n">
+        <v>44.36</v>
+      </c>
+      <c r="I340" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J340" t="inlineStr">
+        <is>
+          <t>09/08/2026 19:36:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>07/08/2026</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>PINTADO</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F341" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G341" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="H341" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="I341" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J341" t="inlineStr">
+        <is>
+          <t>09/08/2026 19:36:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>07/08/2026</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>TAMBAQUI</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F342" s="2" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="G342" s="2" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="H342" s="2" t="n">
+        <v>14.25</v>
+      </c>
+      <c r="I342" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J342" t="inlineStr">
+        <is>
+          <t>09/08/2026 19:36:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>07/08/2026</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F343" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="G343" s="2" t="n">
+        <v>12.24</v>
+      </c>
+      <c r="H343" s="2" t="n">
+        <v>12.43</v>
+      </c>
+      <c r="I343" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J343" t="inlineStr">
+        <is>
+          <t>09/08/2026 19:36:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>07/08/2026</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>TRUTA</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F344" s="2" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="G344" s="2" t="n">
+        <v>38.25</v>
+      </c>
+      <c r="H344" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="I344" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J344" t="inlineStr">
+        <is>
+          <t>09/08/2026 19:36:27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J339"/>
+  <autoFilter ref="A1:J344"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -15453,7 +15673,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -15477,27 +15697,27 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>42.27</v>
+        <v>42.61</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>42.84</v>
+        <v>43.48</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>43.41</v>
+        <v>44.36</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>06/08/2026 10:51:43</t>
+          <t>09/08/2026 19:36:27</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -15524,24 +15744,24 @@
         <v>25</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>25.5</v>
+        <v>26</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>06/08/2026 10:51:43</t>
+          <t>09/08/2026 19:36:27</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -15565,27 +15785,27 @@
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>12</v>
+        <v>13.5</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>12.5</v>
+        <v>13.9</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>13</v>
+        <v>14.25</v>
       </c>
       <c r="I4" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>06/08/2026 10:51:43</t>
+          <t>09/08/2026 19:36:27</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -15609,27 +15829,27 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>11.93</v>
+        <v>12</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>12.22</v>
+        <v>12.24</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>12.45</v>
+        <v>12.43</v>
       </c>
       <c r="I5" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>06/08/2026 10:51:43</t>
+          <t>09/08/2026 19:36:27</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -15666,7 +15886,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>06/08/2026 10:51:43</t>
+          <t>09/08/2026 19:36:27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cotacoes CEAGESP - coleta de 11/08/2026 09:46
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$344</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$349</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J344"/>
+  <dimension ref="A1:J349"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -15591,8 +15591,228 @@
         </is>
       </c>
     </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>10/08/2026</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>FILE DE TILAPIA</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F345" s="2" t="n">
+        <v>42.75</v>
+      </c>
+      <c r="G345" s="2" t="n">
+        <v>43.65</v>
+      </c>
+      <c r="H345" s="2" t="n">
+        <v>44.58</v>
+      </c>
+      <c r="I345" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J345" t="inlineStr">
+        <is>
+          <t>11/08/2026 09:46:44</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>10/08/2026</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>PINTADO</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F346" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G346" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="H346" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="I346" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J346" t="inlineStr">
+        <is>
+          <t>11/08/2026 09:46:44</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>10/08/2026</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>TAMBAQUI</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F347" s="2" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="G347" s="2" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="H347" s="2" t="n">
+        <v>14.25</v>
+      </c>
+      <c r="I347" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J347" t="inlineStr">
+        <is>
+          <t>11/08/2026 09:46:44</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>10/08/2026</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F348" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="G348" s="2" t="n">
+        <v>12.24</v>
+      </c>
+      <c r="H348" s="2" t="n">
+        <v>12.43</v>
+      </c>
+      <c r="I348" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J348" t="inlineStr">
+        <is>
+          <t>11/08/2026 09:46:44</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>10/08/2026</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>TRUTA</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F349" s="2" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="G349" s="2" t="n">
+        <v>38.25</v>
+      </c>
+      <c r="H349" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="I349" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J349" t="inlineStr">
+        <is>
+          <t>11/08/2026 09:46:44</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J344"/>
+  <autoFilter ref="A1:J349"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -15673,7 +15893,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -15697,27 +15917,27 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>42.61</v>
+        <v>42.75</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>43.48</v>
+        <v>43.65</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>44.36</v>
+        <v>44.58</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>09/08/2026 19:36:27</t>
+          <t>11/08/2026 09:46:44</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -15754,14 +15974,14 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>09/08/2026 19:36:27</t>
+          <t>11/08/2026 09:46:44</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -15798,14 +16018,14 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>09/08/2026 19:36:27</t>
+          <t>11/08/2026 09:46:44</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -15842,14 +16062,14 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>09/08/2026 19:36:27</t>
+          <t>11/08/2026 09:46:44</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -15886,7 +16106,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>09/08/2026 19:36:27</t>
+          <t>11/08/2026 09:46:44</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cotacoes CEAGESP - coleta de 13/08/2026 01:41
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$349</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$353</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J349"/>
+  <dimension ref="A1:J353"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -15811,8 +15811,184 @@
         </is>
       </c>
     </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>12/08/2026</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>FILE DE TILAPIA</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F350" s="2" t="n">
+        <v>40.89</v>
+      </c>
+      <c r="G350" s="2" t="n">
+        <v>41.57</v>
+      </c>
+      <c r="H350" s="2" t="n">
+        <v>42.28</v>
+      </c>
+      <c r="I350" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J350" t="inlineStr">
+        <is>
+          <t>13/08/2026 01:41:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>12/08/2026</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>PINTADO</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F351" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="G351" s="2" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="H351" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="I351" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J351" t="inlineStr">
+        <is>
+          <t>13/08/2026 01:41:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>12/08/2026</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>TAMBAQUI</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F352" s="2" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="G352" s="2" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="H352" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="I352" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J352" t="inlineStr">
+        <is>
+          <t>13/08/2026 01:41:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>12/08/2026</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F353" s="2" t="n">
+        <v>12.71</v>
+      </c>
+      <c r="G353" s="2" t="n">
+        <v>12.94</v>
+      </c>
+      <c r="H353" s="2" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="I353" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J353" t="inlineStr">
+        <is>
+          <t>13/08/2026 01:41:14</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J349"/>
+  <autoFilter ref="A1:J353"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -15823,7 +15999,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -15893,7 +16069,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>10/08/2026</t>
+          <t>12/08/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -15917,27 +16093,27 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>42.75</v>
+        <v>40.89</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>43.65</v>
+        <v>41.57</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>44.58</v>
+        <v>42.28</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>11/08/2026 09:46:44</t>
+          <t>13/08/2026 01:41:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>10/08/2026</t>
+          <t>12/08/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -15961,27 +16137,27 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>26</v>
+        <v>27.5</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>11/08/2026 09:46:44</t>
+          <t>13/08/2026 01:41:14</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>10/08/2026</t>
+          <t>12/08/2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -16005,27 +16181,27 @@
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>13.5</v>
+        <v>12.5</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>13.9</v>
+        <v>12.7</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>14.25</v>
+        <v>13</v>
       </c>
       <c r="I4" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>11/08/2026 09:46:44</t>
+          <t>13/08/2026 01:41:14</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>10/08/2026</t>
+          <t>12/08/2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -16049,69 +16225,25 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>12</v>
+        <v>12.71</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>12.24</v>
+        <v>12.94</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>12.43</v>
+        <v>13.2</v>
       </c>
       <c r="I5" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>11/08/2026 09:46:44</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>10/08/2026</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>PESCADOS</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>TRUTA</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>37.5</v>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>38.25</v>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>39</v>
-      </c>
-      <c r="I6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>11/08/2026 09:46:44</t>
+          <t>13/08/2026 01:41:14</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J6"/>
+  <autoFilter ref="A1:J5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Cotacoes CEAGESP - coleta de 15/08/2026 09:22
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$353</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$357</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J353"/>
+  <dimension ref="A1:J357"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -15987,8 +15987,184 @@
         </is>
       </c>
     </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>14/08/2026</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>FILE DE TILAPIA</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F354" s="2" t="n">
+        <v>41.3</v>
+      </c>
+      <c r="G354" s="2" t="n">
+        <v>42.02</v>
+      </c>
+      <c r="H354" s="2" t="n">
+        <v>42.74</v>
+      </c>
+      <c r="I354" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J354" t="inlineStr">
+        <is>
+          <t>15/08/2026 09:22:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>14/08/2026</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>PINTADO</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F355" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="G355" s="2" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="H355" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="I355" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J355" t="inlineStr">
+        <is>
+          <t>15/08/2026 09:22:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>14/08/2026</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>TAMBAQUI</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F356" s="2" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="G356" s="2" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="H356" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="I356" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J356" t="inlineStr">
+        <is>
+          <t>15/08/2026 09:22:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>14/08/2026</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F357" s="2" t="n">
+        <v>12.71</v>
+      </c>
+      <c r="G357" s="2" t="n">
+        <v>12.94</v>
+      </c>
+      <c r="H357" s="2" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="I357" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J357" t="inlineStr">
+        <is>
+          <t>15/08/2026 09:22:27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J353"/>
+  <autoFilter ref="A1:J357"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -16069,7 +16245,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>12/08/2026</t>
+          <t>14/08/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -16093,27 +16269,27 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>40.89</v>
+        <v>41.3</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>41.57</v>
+        <v>42.02</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>42.28</v>
+        <v>42.74</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>13/08/2026 01:41:14</t>
+          <t>15/08/2026 09:22:27</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>12/08/2026</t>
+          <t>14/08/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -16150,14 +16326,14 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>13/08/2026 01:41:14</t>
+          <t>15/08/2026 09:22:27</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>12/08/2026</t>
+          <t>14/08/2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -16194,14 +16370,14 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>13/08/2026 01:41:14</t>
+          <t>15/08/2026 09:22:27</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>12/08/2026</t>
+          <t>14/08/2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -16238,7 +16414,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>13/08/2026 01:41:14</t>
+          <t>15/08/2026 09:22:27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cotacoes CEAGESP - coleta de 18/08/2026 09:30
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$357</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$363</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J357"/>
+  <dimension ref="A1:J363"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -16163,8 +16163,272 @@
         </is>
       </c>
     </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>17/08/2026</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>FILE DE TILAPIA</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F358" s="2" t="n">
+        <v>40.9</v>
+      </c>
+      <c r="G358" s="2" t="n">
+        <v>41.41</v>
+      </c>
+      <c r="H358" s="2" t="n">
+        <v>41.94</v>
+      </c>
+      <c r="I358" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J358" t="inlineStr">
+        <is>
+          <t>18/08/2026 09:30:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>17/08/2026</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>PANGASIUS</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F359" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="G359" s="2" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="H359" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="I359" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J359" t="inlineStr">
+        <is>
+          <t>18/08/2026 09:30:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>17/08/2026</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>PINTADO</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F360" s="2" t="n">
+        <v>24.86</v>
+      </c>
+      <c r="G360" s="2" t="n">
+        <v>25.09</v>
+      </c>
+      <c r="H360" s="2" t="n">
+        <v>25.43</v>
+      </c>
+      <c r="I360" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J360" t="inlineStr">
+        <is>
+          <t>18/08/2026 09:30:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>17/08/2026</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>TAMBAQUI</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F361" s="2" t="n">
+        <v>11.41</v>
+      </c>
+      <c r="G361" s="2" t="n">
+        <v>11.58</v>
+      </c>
+      <c r="H361" s="2" t="n">
+        <v>11.73</v>
+      </c>
+      <c r="I361" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J361" t="inlineStr">
+        <is>
+          <t>18/08/2026 09:30:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>17/08/2026</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F362" s="2" t="n">
+        <v>12.07</v>
+      </c>
+      <c r="G362" s="2" t="n">
+        <v>12.26</v>
+      </c>
+      <c r="H362" s="2" t="n">
+        <v>12.44</v>
+      </c>
+      <c r="I362" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J362" t="inlineStr">
+        <is>
+          <t>18/08/2026 09:30:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>17/08/2026</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>TRUTA</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F363" s="2" t="n">
+        <v>37.43</v>
+      </c>
+      <c r="G363" s="2" t="n">
+        <v>38.16</v>
+      </c>
+      <c r="H363" s="2" t="n">
+        <v>38.87</v>
+      </c>
+      <c r="I363" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J363" t="inlineStr">
+        <is>
+          <t>18/08/2026 09:30:27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J357"/>
+  <autoFilter ref="A1:J363"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -16175,7 +16439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -16245,7 +16509,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>14/08/2026</t>
+          <t>17/08/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -16269,27 +16533,27 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>41.3</v>
+        <v>40.9</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>42.02</v>
+        <v>41.41</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>42.74</v>
+        <v>41.94</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>15/08/2026 09:22:27</t>
+          <t>18/08/2026 09:30:27</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>14/08/2026</t>
+          <t>17/08/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -16299,7 +16563,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>PINTADO</t>
+          <t>PANGASIUS</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -16313,27 +16577,27 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>27.5</v>
+        <v>9.5</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>15/08/2026 09:22:27</t>
+          <t>18/08/2026 09:30:27</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>14/08/2026</t>
+          <t>17/08/2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -16343,7 +16607,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>TAMBAQUI</t>
+          <t>PINTADO</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -16357,27 +16621,27 @@
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>12.5</v>
+        <v>24.86</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>12.7</v>
+        <v>25.09</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>13</v>
+        <v>25.43</v>
       </c>
       <c r="I4" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>15/08/2026 09:22:27</t>
+          <t>18/08/2026 09:30:27</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>14/08/2026</t>
+          <t>17/08/2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -16387,39 +16651,127 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>TAMBAQUI</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>11.41</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>11.58</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>11.73</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>18/08/2026 09:30:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>17/08/2026</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>TILÁPIA</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="n">
-        <v>12.71</v>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>12.94</v>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>13.2</v>
-      </c>
-      <c r="I5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>15/08/2026 09:22:27</t>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>12.07</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>12.26</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>12.44</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>18/08/2026 09:30:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>17/08/2026</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>TRUTA</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>37.43</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>38.16</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>38.87</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>18/08/2026 09:30:27</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J5"/>
+  <autoFilter ref="A1:J7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Cotacoes CEAGESP - coleta de 20/08/2026 09:33
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$363</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$366</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J363"/>
+  <dimension ref="A1:J366"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -16427,8 +16427,140 @@
         </is>
       </c>
     </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>19/08/2026</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>FILE DE TILAPIA</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F364" s="2" t="n">
+        <v>42.04</v>
+      </c>
+      <c r="G364" s="2" t="n">
+        <v>42.7</v>
+      </c>
+      <c r="H364" s="2" t="n">
+        <v>43.36</v>
+      </c>
+      <c r="I364" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J364" t="inlineStr">
+        <is>
+          <t>20/08/2026 09:33:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>19/08/2026</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F365" s="2" t="n">
+        <v>12.29</v>
+      </c>
+      <c r="G365" s="2" t="n">
+        <v>12.43</v>
+      </c>
+      <c r="H365" s="2" t="n">
+        <v>12.59</v>
+      </c>
+      <c r="I365" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J365" t="inlineStr">
+        <is>
+          <t>20/08/2026 09:33:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>19/08/2026</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>TRUTA</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F366" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="G366" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="H366" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="I366" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J366" t="inlineStr">
+        <is>
+          <t>20/08/2026 09:33:19</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J363"/>
+  <autoFilter ref="A1:J366"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -16439,7 +16571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -16509,7 +16641,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>17/08/2026</t>
+          <t>19/08/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -16533,27 +16665,27 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>40.9</v>
+        <v>42.04</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>41.41</v>
+        <v>42.7</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>41.94</v>
+        <v>43.36</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>18/08/2026 09:30:27</t>
+          <t>20/08/2026 09:33:19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>17/08/2026</t>
+          <t>19/08/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -16563,7 +16695,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>PANGASIUS</t>
+          <t>TILÁPIA</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -16577,27 +16709,27 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>9</v>
+        <v>12.29</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>9.5</v>
+        <v>12.43</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>10</v>
+        <v>12.59</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>18/08/2026 09:30:27</t>
+          <t>20/08/2026 09:33:19</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>17/08/2026</t>
+          <t>19/08/2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -16607,7 +16739,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>PINTADO</t>
+          <t>TRUTA</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -16621,157 +16753,25 @@
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>24.86</v>
+        <v>38</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>25.09</v>
+        <v>39</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>25.43</v>
+        <v>40</v>
       </c>
       <c r="I4" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>18/08/2026 09:30:27</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>17/08/2026</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>PESCADOS</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>TAMBAQUI</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="n">
-        <v>11.41</v>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>11.58</v>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>11.73</v>
-      </c>
-      <c r="I5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>18/08/2026 09:30:27</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>17/08/2026</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>PESCADOS</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>TILÁPIA</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>12.07</v>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>12.26</v>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>12.44</v>
-      </c>
-      <c r="I6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>18/08/2026 09:30:27</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>17/08/2026</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>PESCADOS</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>TRUTA</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="n">
-        <v>37.43</v>
-      </c>
-      <c r="G7" s="2" t="n">
-        <v>38.16</v>
-      </c>
-      <c r="H7" s="2" t="n">
-        <v>38.87</v>
-      </c>
-      <c r="I7" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>18/08/2026 09:30:27</t>
+          <t>20/08/2026 09:33:19</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J7"/>
+  <autoFilter ref="A1:J4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Cotacoes CEAGESP - coleta de 22/08/2026 09:24
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$366</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$371</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J366"/>
+  <dimension ref="A1:J371"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -16559,8 +16559,228 @@
         </is>
       </c>
     </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>FILE DE TILAPIA</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F367" s="2" t="n">
+        <v>41.64</v>
+      </c>
+      <c r="G367" s="2" t="n">
+        <v>42.12</v>
+      </c>
+      <c r="H367" s="2" t="n">
+        <v>42.54</v>
+      </c>
+      <c r="I367" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J367" t="inlineStr">
+        <is>
+          <t>22/08/2026 09:23:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>PINTADO</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F368" s="2" t="n">
+        <v>25.34</v>
+      </c>
+      <c r="G368" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="H368" s="2" t="n">
+        <v>26.66</v>
+      </c>
+      <c r="I368" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J368" t="inlineStr">
+        <is>
+          <t>22/08/2026 09:23:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>TAMBAQUI</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F369" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="G369" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="H369" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I369" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J369" t="inlineStr">
+        <is>
+          <t>22/08/2026 09:23:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F370" s="2" t="n">
+        <v>11.57</v>
+      </c>
+      <c r="G370" s="2" t="n">
+        <v>11.98</v>
+      </c>
+      <c r="H370" s="2" t="n">
+        <v>12.42</v>
+      </c>
+      <c r="I370" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J370" t="inlineStr">
+        <is>
+          <t>22/08/2026 09:23:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>TRUTA</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F371" s="2" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="G371" s="2" t="n">
+        <v>38.25</v>
+      </c>
+      <c r="H371" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="I371" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J371" t="inlineStr">
+        <is>
+          <t>22/08/2026 09:23:58</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J366"/>
+  <autoFilter ref="A1:J371"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -16571,7 +16791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -16641,7 +16861,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>19/08/2026</t>
+          <t>21/08/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -16665,27 +16885,27 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>42.04</v>
+        <v>41.64</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>42.7</v>
+        <v>42.12</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>43.36</v>
+        <v>42.54</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>20/08/2026 09:33:19</t>
+          <t>22/08/2026 09:23:58</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>19/08/2026</t>
+          <t>21/08/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -16695,7 +16915,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>TILÁPIA</t>
+          <t>PINTADO</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -16709,27 +16929,27 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>12.29</v>
+        <v>25.34</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>12.43</v>
+        <v>26</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>12.59</v>
+        <v>26.66</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>20/08/2026 09:33:19</t>
+          <t>22/08/2026 09:23:58</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>19/08/2026</t>
+          <t>21/08/2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -16739,39 +16959,127 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>TAMBAQUI</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>22/08/2026 09:23:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>11.57</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>11.98</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>12.42</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>22/08/2026 09:23:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>TRUTA</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="n">
-        <v>38</v>
-      </c>
-      <c r="G4" s="2" t="n">
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>38.25</v>
+      </c>
+      <c r="H6" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="H4" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="I4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>20/08/2026 09:33:19</t>
+      <c r="I6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>22/08/2026 09:23:58</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J4"/>
+  <autoFilter ref="A1:J6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Cotacoes CEAGESP - coleta de 25/08/2026 09:33
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$371</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$375</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J371"/>
+  <dimension ref="A1:J375"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -16779,8 +16779,184 @@
         </is>
       </c>
     </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>FILE DE TILAPIA</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F372" s="2" t="n">
+        <v>41.16</v>
+      </c>
+      <c r="G372" s="2" t="n">
+        <v>41.7</v>
+      </c>
+      <c r="H372" s="2" t="n">
+        <v>42.25</v>
+      </c>
+      <c r="I372" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J372" t="inlineStr">
+        <is>
+          <t>25/08/2026 09:33:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>TAMBAQUI</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F373" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="G373" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="H373" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I373" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J373" t="inlineStr">
+        <is>
+          <t>25/08/2026 09:33:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F374" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="G374" s="2" t="n">
+        <v>12.32</v>
+      </c>
+      <c r="H374" s="2" t="n">
+        <v>12.56</v>
+      </c>
+      <c r="I374" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J374" t="inlineStr">
+        <is>
+          <t>25/08/2026 09:33:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>TRUTA</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F375" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="G375" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="H375" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="I375" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J375" t="inlineStr">
+        <is>
+          <t>25/08/2026 09:33:50</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J371"/>
+  <autoFilter ref="A1:J375"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -16791,7 +16967,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -16861,7 +17037,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>21/08/2026</t>
+          <t>24/08/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -16885,27 +17061,27 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>41.64</v>
+        <v>41.16</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>42.12</v>
+        <v>41.7</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>42.54</v>
+        <v>42.25</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>22/08/2026 09:23:58</t>
+          <t>25/08/2026 09:33:50</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>21/08/2026</t>
+          <t>24/08/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -16915,7 +17091,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>PINTADO</t>
+          <t>TAMBAQUI</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -16929,27 +17105,27 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>25.34</v>
+        <v>13</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>26.66</v>
+        <v>15</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>22/08/2026 09:23:58</t>
+          <t>25/08/2026 09:33:50</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>21/08/2026</t>
+          <t>24/08/2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -16959,7 +17135,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>TAMBAQUI</t>
+          <t>TILÁPIA</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -16973,27 +17149,27 @@
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>14</v>
+        <v>12.32</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>15</v>
+        <v>12.56</v>
       </c>
       <c r="I4" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>22/08/2026 09:23:58</t>
+          <t>25/08/2026 09:33:50</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>21/08/2026</t>
+          <t>24/08/2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -17003,7 +17179,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>TILÁPIA</t>
+          <t>TRUTA</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -17017,69 +17193,25 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>11.57</v>
+        <v>38</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>11.98</v>
+        <v>39</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>12.42</v>
+        <v>40</v>
       </c>
       <c r="I5" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>22/08/2026 09:23:58</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>21/08/2026</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>PESCADOS</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>TRUTA</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>37.5</v>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>38.25</v>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>39</v>
-      </c>
-      <c r="I6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>22/08/2026 09:23:58</t>
+          <t>25/08/2026 09:33:50</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J6"/>
+  <autoFilter ref="A1:J5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Cotacoes CEAGESP - coleta de 27/08/2026 16:10
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$375</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$378</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J375"/>
+  <dimension ref="A1:J378"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -16955,8 +16955,140 @@
         </is>
       </c>
     </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>26/08/2026</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>FILE DE TILAPIA</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F376" s="2" t="n">
+        <v>41.08</v>
+      </c>
+      <c r="G376" s="2" t="n">
+        <v>41.62</v>
+      </c>
+      <c r="H376" s="2" t="n">
+        <v>42.16</v>
+      </c>
+      <c r="I376" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J376" t="inlineStr">
+        <is>
+          <t>27/08/2026 16:10:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>26/08/2026</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F377" s="2" t="n">
+        <v>12.25</v>
+      </c>
+      <c r="G377" s="2" t="n">
+        <v>12.42</v>
+      </c>
+      <c r="H377" s="2" t="n">
+        <v>12.57</v>
+      </c>
+      <c r="I377" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J377" t="inlineStr">
+        <is>
+          <t>27/08/2026 16:10:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>26/08/2026</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>TRUTA</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F378" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="G378" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="H378" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="I378" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J378" t="inlineStr">
+        <is>
+          <t>27/08/2026 16:10:39</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J375"/>
+  <autoFilter ref="A1:J378"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -16967,7 +17099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -17037,7 +17169,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>24/08/2026</t>
+          <t>26/08/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -17061,27 +17193,27 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>41.16</v>
+        <v>41.08</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>41.7</v>
+        <v>41.62</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>42.25</v>
+        <v>42.16</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>25/08/2026 09:33:50</t>
+          <t>27/08/2026 16:10:39</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>24/08/2026</t>
+          <t>26/08/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -17091,7 +17223,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>TAMBAQUI</t>
+          <t>TILÁPIA</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -17105,27 +17237,27 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>13</v>
+        <v>12.25</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>14</v>
+        <v>12.42</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>15</v>
+        <v>12.57</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>25/08/2026 09:33:50</t>
+          <t>27/08/2026 16:10:39</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>24/08/2026</t>
+          <t>26/08/2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -17135,7 +17267,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>TILÁPIA</t>
+          <t>TRUTA</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -17149,69 +17281,25 @@
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>12</v>
+        <v>38</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>12.32</v>
+        <v>39</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>12.56</v>
+        <v>40</v>
       </c>
       <c r="I4" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>25/08/2026 09:33:50</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>24/08/2026</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>PESCADOS</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>TRUTA</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="n">
-        <v>38</v>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>39</v>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="I5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>25/08/2026 09:33:50</t>
+          <t>27/08/2026 16:10:39</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J5"/>
+  <autoFilter ref="A1:J4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Cotacoes CEAGESP - coleta de 29/08/2026 00:07
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$378</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$384</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J378"/>
+  <dimension ref="A1:J384"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -17087,8 +17087,272 @@
         </is>
       </c>
     </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>FILE DE TILAPIA</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F379" s="2" t="n">
+        <v>41.14</v>
+      </c>
+      <c r="G379" s="2" t="n">
+        <v>42.13</v>
+      </c>
+      <c r="H379" s="2" t="n">
+        <v>43.31</v>
+      </c>
+      <c r="I379" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J379" t="inlineStr">
+        <is>
+          <t>29/08/2026 00:07:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>PANGASIUS</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F380" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="G380" s="2" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="H380" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="I380" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J380" t="inlineStr">
+        <is>
+          <t>29/08/2026 00:07:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>PINTADO</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F381" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="G381" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="H381" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="I381" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J381" t="inlineStr">
+        <is>
+          <t>29/08/2026 00:07:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>TAMBAQUI</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F382" s="2" t="n">
+        <v>14.27</v>
+      </c>
+      <c r="G382" s="2" t="n">
+        <v>15.27</v>
+      </c>
+      <c r="H382" s="2" t="n">
+        <v>15.45</v>
+      </c>
+      <c r="I382" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J382" t="inlineStr">
+        <is>
+          <t>29/08/2026 00:07:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F383" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G383" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="H383" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="I383" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J383" t="inlineStr">
+        <is>
+          <t>29/08/2026 00:07:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>TRUTA</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F384" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="G384" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="H384" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="I384" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J384" t="inlineStr">
+        <is>
+          <t>29/08/2026 00:07:09</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J378"/>
+  <autoFilter ref="A1:J384"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17099,7 +17363,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -17169,7 +17433,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>28/08/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -17193,27 +17457,27 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>41.08</v>
+        <v>41.14</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>41.62</v>
+        <v>42.13</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>42.16</v>
+        <v>43.31</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>27/08/2026 16:10:39</t>
+          <t>29/08/2026 00:07:09</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>28/08/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -17223,7 +17487,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>TILÁPIA</t>
+          <t>PANGASIUS</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -17237,27 +17501,27 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>12.25</v>
+        <v>9</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>12.42</v>
+        <v>9.5</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>12.57</v>
+        <v>10</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>27/08/2026 16:10:39</t>
+          <t>29/08/2026 00:07:09</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>28/08/2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -17267,39 +17531,171 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>PINTADO</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>29/08/2026 00:07:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>TAMBAQUI</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>14.27</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>15.27</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>15.45</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>29/08/2026 00:07:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>29/08/2026 00:07:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>TRUTA</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="n">
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="G7" s="2" t="n">
         <v>38</v>
       </c>
-      <c r="G4" s="2" t="n">
-        <v>39</v>
-      </c>
-      <c r="H4" s="2" t="n">
+      <c r="H7" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="I4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>27/08/2026 16:10:39</t>
+      <c r="I7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>29/08/2026 00:07:09</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J4"/>
+  <autoFilter ref="A1:J7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Cotacoes CEAGESP - coleta de 31/08/2026 21:29
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$384</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$387</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J384"/>
+  <dimension ref="A1:J387"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -17351,8 +17351,140 @@
         </is>
       </c>
     </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>FILE DE TILAPIA</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F385" s="2" t="n">
+        <v>40.97</v>
+      </c>
+      <c r="G385" s="2" t="n">
+        <v>41.94</v>
+      </c>
+      <c r="H385" s="2" t="n">
+        <v>42.89</v>
+      </c>
+      <c r="I385" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J385" t="inlineStr">
+        <is>
+          <t>31/08/2026 21:29:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F386" s="2" t="n">
+        <v>11.99</v>
+      </c>
+      <c r="G386" s="2" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="H386" s="2" t="n">
+        <v>12.78</v>
+      </c>
+      <c r="I386" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J386" t="inlineStr">
+        <is>
+          <t>31/08/2026 21:29:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>TRUTA</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F387" s="2" t="n">
+        <v>37.8</v>
+      </c>
+      <c r="G387" s="2" t="n">
+        <v>38.7</v>
+      </c>
+      <c r="H387" s="2" t="n">
+        <v>39.6</v>
+      </c>
+      <c r="I387" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J387" t="inlineStr">
+        <is>
+          <t>31/08/2026 21:29:41</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J384"/>
+  <autoFilter ref="A1:J387"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17363,7 +17495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -17433,7 +17565,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>28/08/2026</t>
+          <t>31/08/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -17457,27 +17589,27 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>41.14</v>
+        <v>40.97</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>42.13</v>
+        <v>41.94</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>43.31</v>
+        <v>42.89</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>29/08/2026 00:07:09</t>
+          <t>31/08/2026 21:29:41</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>28/08/2026</t>
+          <t>31/08/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -17487,7 +17619,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>PANGASIUS</t>
+          <t>TILÁPIA</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -17501,27 +17633,27 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>9</v>
+        <v>11.99</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>9.5</v>
+        <v>12.4</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>10</v>
+        <v>12.78</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>29/08/2026 00:07:09</t>
+          <t>31/08/2026 21:29:41</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>28/08/2026</t>
+          <t>31/08/2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -17531,7 +17663,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>PINTADO</t>
+          <t>TRUTA</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -17545,157 +17677,25 @@
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>22</v>
+        <v>37.8</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>23</v>
+        <v>38.7</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>24</v>
+        <v>39.6</v>
       </c>
       <c r="I4" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>29/08/2026 00:07:09</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>28/08/2026</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>PESCADOS</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>TAMBAQUI</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="n">
-        <v>14.27</v>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>15.27</v>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>15.45</v>
-      </c>
-      <c r="I5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>29/08/2026 00:07:09</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>28/08/2026</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>PESCADOS</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>TILÁPIA</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="I6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>29/08/2026 00:07:09</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>28/08/2026</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>PESCADOS</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>TRUTA</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="G7" s="2" t="n">
-        <v>38</v>
-      </c>
-      <c r="H7" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="I7" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>29/08/2026 00:07:09</t>
+          <t>31/08/2026 21:29:41</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J7"/>
+  <autoFilter ref="A1:J4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Cotacoes CEAGESP - coleta de 02/09/2026 17:51
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$387</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$389</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J387"/>
+  <dimension ref="A1:J389"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -17483,8 +17483,96 @@
         </is>
       </c>
     </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>FILE DE TILAPIA</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F388" s="2" t="n">
+        <v>42.86</v>
+      </c>
+      <c r="G388" s="2" t="n">
+        <v>43.8</v>
+      </c>
+      <c r="H388" s="2" t="n">
+        <v>44.74</v>
+      </c>
+      <c r="I388" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J388" t="inlineStr">
+        <is>
+          <t>02/09/2026 17:51:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F389" s="2" t="n">
+        <v>12.04</v>
+      </c>
+      <c r="G389" s="2" t="n">
+        <v>12.55</v>
+      </c>
+      <c r="H389" s="2" t="n">
+        <v>13.02</v>
+      </c>
+      <c r="I389" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J389" t="inlineStr">
+        <is>
+          <t>02/09/2026 17:51:13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J387"/>
+  <autoFilter ref="A1:J389"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17495,7 +17583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -17565,7 +17653,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>31/08/2026</t>
+          <t>02/09/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -17589,27 +17677,27 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>40.97</v>
+        <v>42.86</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>41.94</v>
+        <v>43.8</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>42.89</v>
+        <v>44.74</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>31/08/2026 21:29:41</t>
+          <t>02/09/2026 17:51:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>31/08/2026</t>
+          <t>02/09/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -17633,69 +17721,25 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>11.99</v>
+        <v>12.04</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>12.4</v>
+        <v>12.55</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>12.78</v>
+        <v>13.02</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>31/08/2026 21:29:41</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>31/08/2026</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>PESCADOS</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>TRUTA</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="n">
-        <v>37.8</v>
-      </c>
-      <c r="G4" s="2" t="n">
-        <v>38.7</v>
-      </c>
-      <c r="H4" s="2" t="n">
-        <v>39.6</v>
-      </c>
-      <c r="I4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>31/08/2026 21:29:41</t>
+          <t>02/09/2026 17:51:13</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J4"/>
+  <autoFilter ref="A1:J3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Cotacoes CEAGESP - coleta de 04/09/2026 19:55
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$389</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$393</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J389"/>
+  <dimension ref="A1:J393"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -17571,8 +17571,184 @@
         </is>
       </c>
     </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>04/09/2026</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>FILE DE TILAPIA</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F390" s="2" t="n">
+        <v>40.75</v>
+      </c>
+      <c r="G390" s="2" t="n">
+        <v>41.35</v>
+      </c>
+      <c r="H390" s="2" t="n">
+        <v>41.96</v>
+      </c>
+      <c r="I390" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J390" t="inlineStr">
+        <is>
+          <t>04/09/2026 19:55:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>04/09/2026</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>PINTADO</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F391" s="2" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="G391" s="2" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="H391" s="2" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="I391" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J391" t="inlineStr">
+        <is>
+          <t>04/09/2026 19:55:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>04/09/2026</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>TAMBAQUI</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F392" s="2" t="n">
+        <v>12.99</v>
+      </c>
+      <c r="G392" s="2" t="n">
+        <v>13.77</v>
+      </c>
+      <c r="H392" s="2" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="I392" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J392" t="inlineStr">
+        <is>
+          <t>04/09/2026 19:55:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>04/09/2026</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F393" s="2" t="n">
+        <v>11.87</v>
+      </c>
+      <c r="G393" s="2" t="n">
+        <v>12.29</v>
+      </c>
+      <c r="H393" s="2" t="n">
+        <v>12.74</v>
+      </c>
+      <c r="I393" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J393" t="inlineStr">
+        <is>
+          <t>04/09/2026 19:55:03</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J389"/>
+  <autoFilter ref="A1:J393"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17583,7 +17759,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -17653,7 +17829,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>02/09/2026</t>
+          <t>04/09/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -17677,27 +17853,27 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>42.86</v>
+        <v>40.75</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>43.8</v>
+        <v>41.35</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>44.74</v>
+        <v>41.96</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>02/09/2026 17:51:13</t>
+          <t>04/09/2026 19:55:03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>02/09/2026</t>
+          <t>04/09/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -17707,39 +17883,127 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>PINTADO</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>04/09/2026 19:55:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>04/09/2026</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>TAMBAQUI</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>12.99</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>13.77</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>04/09/2026 19:55:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>04/09/2026</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>TILÁPIA</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="n">
-        <v>12.04</v>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>12.55</v>
-      </c>
-      <c r="H3" s="2" t="n">
-        <v>13.02</v>
-      </c>
-      <c r="I3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>02/09/2026 17:51:13</t>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>11.87</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>12.29</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>12.74</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>04/09/2026 19:55:03</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J3"/>
+  <autoFilter ref="A1:J5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>